<commit_message>
Record failure log from smoke-test run (5 venues now correctly flagged)
Live run against all venue sites confirms the fix: McGuffie's Live,
Lou Lou's Jungle Room, Humphrey's Concerts, 710 Beach Club, and
Worldbeat Center all previously reported "0 events" silently in the
summary. With this change they're retried and, still empty, logged
as NoEventsFound failures instead.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,6 +441,131 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Last Failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>710 Beach Club</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Humphrey's Concerts</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lou Lou's Jungle Room</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>McGuffie's Live</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Worldbeat Center</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Thu 09/03/2026 17:33)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -461,11 +461,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:25</t>
+          <t>2026-09-03 17:31</t>
         </is>
       </c>
     </row>
@@ -486,11 +486,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:25</t>
+          <t>2026-09-03 17:31</t>
         </is>
       </c>
     </row>
@@ -511,11 +511,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:25</t>
+          <t>2026-09-03 17:31</t>
         </is>
       </c>
     </row>
@@ -536,11 +536,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:25</t>
+          <t>2026-09-03 17:31</t>
         </is>
       </c>
     </row>
@@ -561,11 +561,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:25</t>
+          <t>2026-09-03 17:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Thu 09/03/2026 17:36)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -461,11 +461,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:31</t>
+          <t>2026-09-03 17:35</t>
         </is>
       </c>
     </row>
@@ -486,11 +486,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:31</t>
+          <t>2026-09-03 17:35</t>
         </is>
       </c>
     </row>
@@ -511,11 +511,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:31</t>
+          <t>2026-09-03 17:35</t>
         </is>
       </c>
     </row>
@@ -536,11 +536,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:31</t>
+          <t>2026-09-03 17:35</t>
         </is>
       </c>
     </row>
@@ -561,11 +561,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:31</t>
+          <t>2026-09-03 17:35</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,6 +610,131 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>710 Beach Club</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Humphrey's Concerts</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lou Lou's Jungle Room</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>McGuffie's Live</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Worldbeat Center</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NoEventsFound</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>scraper returned 0 events</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:35</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refresh event data (Thu 09/03/2026 17:38)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -461,11 +461,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -486,11 +486,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -511,11 +511,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -536,11 +536,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -561,11 +561,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -627,11 +627,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -652,11 +652,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -677,11 +677,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -702,11 +702,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:35</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Thu 09/03/2026 17:42)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -461,11 +461,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -486,11 +486,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -511,11 +511,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -536,11 +536,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -561,11 +561,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -627,11 +627,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -652,11 +652,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -677,11 +677,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -702,11 +702,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Thu 09/03/2026 17:44)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -461,11 +461,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -486,11 +486,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -511,11 +511,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -536,11 +536,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -561,11 +561,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -627,11 +627,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -652,11 +652,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -677,11 +677,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -702,11 +702,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-03 17:41</t>
+          <t>2026-09-03 17:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update stale comment; record failure log from validation run
- build_events_data.py: fix the SCRAPERS comment above loulous/
  humphreys/quartyard, which was stale after this branch's scraper
  fixes (Lou Lou's now fetches its own casbahmusic.com page, and
  Humphrey's moved off casbahmusic.com entirely).
- Committed failure_log.xlsx from a live validation run confirming
  McGuffie's Live, Lou Lou's Jungle Room, and Humphrey's Concerts are
  fixed (dropped out of the log entirely), while 710 Beach Club and
  Worldbeat Center remain (as expected - see commit history for why).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,18 +461,18 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:43</t>
+          <t>2026-09-03 17:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Humphrey's Concerts</t>
+          <t>Worldbeat Center</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -486,86 +486,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Lou Lou's Jungle Room</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>NoEventsFound</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>scraper returned 0 events</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-09-03 17:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>McGuffie's Live</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>NoEventsFound</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>scraper returned 0 events</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-09-03 17:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Worldbeat Center</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>NoEventsFound</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>scraper returned 0 events</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-09-03 17:43</t>
+          <t>2026-09-03 17:58</t>
         </is>
       </c>
     </row>
@@ -580,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -627,18 +552,18 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-03 17:43</t>
+          <t>2026-09-03 17:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Humphrey's Concerts</t>
+          <t>Worldbeat Center</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -652,86 +577,11 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-03 17:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Lou Lou's Jungle Room</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>NoEventsFound</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>scraper returned 0 events</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-09-03 17:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>McGuffie's Live</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>NoEventsFound</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>scraper returned 0 events</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-09-03 17:43</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Worldbeat Center</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>NoEventsFound</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>scraper returned 0 events</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-09-03 17:43</t>
+          <t>2026-09-03 17:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh event data (Fri 09/04/2026  7:33)
Automated data refresh via update-events.bat

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scraper/failure_log.xlsx
+++ b/scraper/failure_log.xlsx
@@ -461,11 +461,11 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-04 07:27</t>
+          <t>2026-09-04 07:31</t>
         </is>
       </c>
     </row>

</xml_diff>